<commit_message>
Update daily stock monitor reports
</commit_message>
<xml_diff>
--- a/data/BOLL/EXCLE/AAOI_1_20260923.xlsx
+++ b/data/BOLL/EXCLE/AAOI_1_20260923.xlsx
@@ -196,12 +196,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'30日跟踪'!$A$8:$A$9</f>
+              <f>'30日跟踪'!$A$8:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'30日跟踪'!$D$8:$D$9</f>
+              <f>'30日跟踪'!$D$8:$D$10</f>
             </numRef>
           </val>
         </ser>
@@ -584,7 +584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="6">
@@ -660,7 +660,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2/30</t>
+          <t>3/30</t>
         </is>
       </c>
     </row>
@@ -728,6 +728,26 @@
       <c r="E9" t="inlineStr">
         <is>
           <t>第2/30个交易日</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>101.4000015258789</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>0.366230576118598</v>
+      </c>
+      <c r="D10" s="6">
+        <f>B10/$B$8-1</f>
+        <v/>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>第3/30个交易日</t>
         </is>
       </c>
     </row>

</xml_diff>